<commit_message>
CH4 dD peak updates
Updated dD backgrounds based on the intensity of the 13C peak
</commit_message>
<xml_diff>
--- a/backgrounds_mean.xlsx
+++ b/backgrounds_mean.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:O19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,47 +467,62 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>i16</t>
+          <t>i28</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>i16_se</t>
+          <t>i28_se</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>i16_std</t>
+          <t>i28_std</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>i17</t>
+          <t>i29</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>i17_se</t>
+          <t>i29_se</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>i17_std</t>
+          <t>i29_std</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>i18</t>
+          <t>i30</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>i18_se</t>
+          <t>i30_se</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>i18_std</t>
+          <t>i30_std</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>i31</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>i31_se</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>i31_std</t>
         </is>
       </c>
     </row>
@@ -522,31 +537,40 @@
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>605.6664980332491</v>
+        <v>-93181.44412426048</v>
       </c>
       <c r="E2" t="n">
-        <v>679.4447545299873</v>
+        <v>2404.65968233168</v>
       </c>
       <c r="F2" t="n">
-        <v>6445.778905706302</v>
+        <v>22812.60478123519</v>
       </c>
       <c r="G2" t="n">
-        <v>-36885.04927295838</v>
+        <v>105.0589658354445</v>
       </c>
       <c r="H2" t="n">
-        <v>77.00484778867268</v>
+        <v>173.6005912359678</v>
       </c>
       <c r="I2" t="n">
-        <v>730.5321296603581</v>
+        <v>1646.91981437257</v>
       </c>
       <c r="J2" t="n">
-        <v>0.1483494060166077</v>
+        <v>-16040.13582703898</v>
       </c>
       <c r="K2" t="n">
-        <v>0.03663815425005915</v>
+        <v>79.1345800695203</v>
       </c>
       <c r="L2" t="n">
-        <v>0.3475800500842957</v>
+        <v>750.7365441019498</v>
+      </c>
+      <c r="M2" t="n">
+        <v>-2181.053453543348</v>
+      </c>
+      <c r="N2" t="n">
+        <v>39.19960801683687</v>
+      </c>
+      <c r="O2" t="n">
+        <v>371.8801341570016</v>
       </c>
     </row>
     <row r="3">
@@ -558,31 +582,40 @@
         <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>-43.94513375798722</v>
+        <v>-89200.58891337585</v>
       </c>
       <c r="E3" t="n">
-        <v>546.8548584978429</v>
+        <v>2657.794856075508</v>
       </c>
       <c r="F3" t="n">
-        <v>5187.920707146806</v>
+        <v>25214.05589603403</v>
       </c>
       <c r="G3" t="n">
-        <v>-37174.24607027951</v>
+        <v>-112.1793985308026</v>
       </c>
       <c r="H3" t="n">
-        <v>94.57254904110506</v>
+        <v>168.0143600746187</v>
       </c>
       <c r="I3" t="n">
-        <v>897.193977293595</v>
+        <v>1593.924172354358</v>
       </c>
       <c r="J3" t="n">
-        <v>0.2966988120332154</v>
+        <v>-16090.51583324917</v>
       </c>
       <c r="K3" t="n">
-        <v>0.06329989937512924</v>
+        <v>76.67464708395607</v>
       </c>
       <c r="L3" t="n">
-        <v>0.6005155730546327</v>
+        <v>727.3995707246665</v>
+      </c>
+      <c r="M3" t="n">
+        <v>-2178.656948296896</v>
+      </c>
+      <c r="N3" t="n">
+        <v>50.96097823974709</v>
+      </c>
+      <c r="O3" t="n">
+        <v>483.4582890836373</v>
       </c>
     </row>
     <row r="4">
@@ -594,31 +627,40 @@
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>638.4444006504698</v>
+        <v>-91591.75508563634</v>
       </c>
       <c r="E4" t="n">
-        <v>533.6271521358781</v>
+        <v>2326.052362059937</v>
       </c>
       <c r="F4" t="n">
-        <v>5062.431666175681</v>
+        <v>22066.87026277209</v>
       </c>
       <c r="G4" t="n">
-        <v>-37108.8464022222</v>
+        <v>-152.4684678162853</v>
       </c>
       <c r="H4" t="n">
-        <v>85.84624812668615</v>
+        <v>197.7700053129828</v>
       </c>
       <c r="I4" t="n">
-        <v>814.4090179808736</v>
+        <v>1876.211008957882</v>
       </c>
       <c r="J4" t="n">
-        <v>0.1483494060166077</v>
+        <v>-16166.17670441434</v>
       </c>
       <c r="K4" t="n">
-        <v>0.03961621344771563</v>
+        <v>77.9789920102147</v>
       </c>
       <c r="L4" t="n">
-        <v>0.3758324002985198</v>
+        <v>739.7736731890515</v>
+      </c>
+      <c r="M4" t="n">
+        <v>-2181.267699594378</v>
+      </c>
+      <c r="N4" t="n">
+        <v>46.30824203177383</v>
+      </c>
+      <c r="O4" t="n">
+        <v>439.3185577762462</v>
       </c>
     </row>
     <row r="5">
@@ -630,31 +672,40 @@
         <v>1</v>
       </c>
       <c r="D5" t="n">
-        <v>0.6821318413783349</v>
+        <v>-91145.05985162592</v>
       </c>
       <c r="E5" t="n">
-        <v>583.5829653061143</v>
+        <v>2057.623397892528</v>
       </c>
       <c r="F5" t="n">
-        <v>5536.354122127031</v>
+        <v>19520.32951258588</v>
       </c>
       <c r="G5" t="n">
-        <v>-36962.25337983412</v>
+        <v>-175.3198783010193</v>
       </c>
       <c r="H5" t="n">
-        <v>87.31129295663381</v>
+        <v>168.019112948223</v>
       </c>
       <c r="I5" t="n">
-        <v>828.3076535915395</v>
+        <v>1593.96926207242</v>
       </c>
       <c r="J5" t="n">
-        <v>0.1589457921606511</v>
+        <v>-16176.26392453986</v>
       </c>
       <c r="K5" t="n">
-        <v>0.04328386158768253</v>
+        <v>68.14635318642796</v>
       </c>
       <c r="L5" t="n">
-        <v>0.4106267656336461</v>
+        <v>646.4930709101561</v>
+      </c>
+      <c r="M5" t="n">
+        <v>-2144.771017875603</v>
+      </c>
+      <c r="N5" t="n">
+        <v>45.60213386645885</v>
+      </c>
+      <c r="O5" t="n">
+        <v>432.6198275457321</v>
       </c>
     </row>
     <row r="6">
@@ -666,31 +717,40 @@
         <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>-459.9484157271024</v>
+        <v>-87571.58677230601</v>
       </c>
       <c r="E6" t="n">
-        <v>638.3718922410829</v>
+        <v>2061.980976391742</v>
       </c>
       <c r="F6" t="n">
-        <v>6056.127521140178</v>
+        <v>19561.66913200737</v>
       </c>
       <c r="G6" t="n">
-        <v>-37118.69150665028</v>
+        <v>-6.38413412273942</v>
       </c>
       <c r="H6" t="n">
-        <v>78.83181152794049</v>
+        <v>176.7523827501823</v>
       </c>
       <c r="I6" t="n">
-        <v>747.8642295162309</v>
+        <v>1676.820334057297</v>
       </c>
       <c r="J6" t="n">
-        <v>0.1589457921606511</v>
+        <v>-16166.78775695443</v>
       </c>
       <c r="K6" t="n">
-        <v>0.04057588757942112</v>
+        <v>75.9494930464641</v>
       </c>
       <c r="L6" t="n">
-        <v>0.3849366685017211</v>
+        <v>720.5201554858413</v>
+      </c>
+      <c r="M6" t="n">
+        <v>-2179.412708320565</v>
+      </c>
+      <c r="N6" t="n">
+        <v>45.40740406244986</v>
+      </c>
+      <c r="O6" t="n">
+        <v>430.7724584187724</v>
       </c>
     </row>
     <row r="7">
@@ -702,31 +762,40 @@
         <v>1</v>
       </c>
       <c r="D7" t="n">
-        <v>121.420879922538</v>
+        <v>-89358.30519520755</v>
       </c>
       <c r="E7" t="n">
-        <v>630.3439212217368</v>
+        <v>2296.274738202108</v>
       </c>
       <c r="F7" t="n">
-        <v>5979.967500907305</v>
+        <v>21784.37491867656</v>
       </c>
       <c r="G7" t="n">
-        <v>-37001.82891410158</v>
+        <v>59.64890937567949</v>
       </c>
       <c r="H7" t="n">
-        <v>87.16806593372119</v>
+        <v>198.7554046906344</v>
       </c>
       <c r="I7" t="n">
-        <v>826.9488827468726</v>
+        <v>1885.559328272755</v>
       </c>
       <c r="J7" t="n">
-        <v>0.1907349505927813</v>
+        <v>-16010.40042889167</v>
       </c>
       <c r="K7" t="n">
-        <v>0.04570807580692174</v>
+        <v>72.26814562699978</v>
       </c>
       <c r="L7" t="n">
-        <v>0.4336248810405341</v>
+        <v>685.5958273741697</v>
+      </c>
+      <c r="M7" t="n">
+        <v>-2142.615394572892</v>
+      </c>
+      <c r="N7" t="n">
+        <v>47.62305532139396</v>
+      </c>
+      <c r="O7" t="n">
+        <v>451.791971855421</v>
       </c>
     </row>
     <row r="8">
@@ -738,31 +807,40 @@
         <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>1231.637936906649</v>
+        <v>-91420.96370239391</v>
       </c>
       <c r="E8" t="n">
-        <v>614.7021772441234</v>
+        <v>2466.207831029958</v>
       </c>
       <c r="F8" t="n">
-        <v>5831.576888267865</v>
+        <v>23396.50178819505</v>
       </c>
       <c r="G8" t="n">
-        <v>-37144.21782202214</v>
+        <v>-102.9940260402075</v>
       </c>
       <c r="H8" t="n">
-        <v>90.00074288428905</v>
+        <v>178.2256059547591</v>
       </c>
       <c r="I8" t="n">
-        <v>853.8220158646366</v>
+        <v>1690.796556542122</v>
       </c>
       <c r="J8" t="n">
-        <v>0.2331205048702451</v>
+        <v>-16114.93107498306</v>
       </c>
       <c r="K8" t="n">
-        <v>0.05287467112692638</v>
+        <v>75.47144450837598</v>
       </c>
       <c r="L8" t="n">
-        <v>0.5016131738802879</v>
+        <v>715.9849888484247</v>
+      </c>
+      <c r="M8" t="n">
+        <v>-2147.445126192348</v>
+      </c>
+      <c r="N8" t="n">
+        <v>45.02667723372544</v>
+      </c>
+      <c r="O8" t="n">
+        <v>427.1605665834663</v>
       </c>
     </row>
     <row r="9">
@@ -774,31 +852,40 @@
         <v>1</v>
       </c>
       <c r="D9" t="n">
-        <v>-797.2312577714069</v>
+        <v>-90356.76970638192</v>
       </c>
       <c r="E9" t="n">
-        <v>568.3298052912328</v>
+        <v>2240.061468794228</v>
       </c>
       <c r="F9" t="n">
-        <v>5391.649940640931</v>
+        <v>21251.08902051586</v>
       </c>
       <c r="G9" t="n">
-        <v>-37160.45534664014</v>
+        <v>-337.9392677307531</v>
       </c>
       <c r="H9" t="n">
-        <v>70.42273851018771</v>
+        <v>189.1377373452632</v>
       </c>
       <c r="I9" t="n">
-        <v>668.0887582759381</v>
+        <v>1794.318124505161</v>
       </c>
       <c r="J9" t="n">
-        <v>0.2331205048702451</v>
+        <v>-16239.47588531192</v>
       </c>
       <c r="K9" t="n">
-        <v>0.05068176028609093</v>
+        <v>77.22360844833025</v>
       </c>
       <c r="L9" t="n">
-        <v>0.480809394992143</v>
+        <v>732.6074755012346</v>
+      </c>
+      <c r="M9" t="n">
+        <v>-2158.524891666192</v>
+      </c>
+      <c r="N9" t="n">
+        <v>51.53155807200751</v>
+      </c>
+      <c r="O9" t="n">
+        <v>488.8712846543366</v>
       </c>
     </row>
     <row r="10">
@@ -810,108 +897,453 @@
         <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>114.8341708870545</v>
+        <v>-90002.08277076477</v>
       </c>
       <c r="E10" t="n">
-        <v>616.3173857127788</v>
+        <v>2423.737486656898</v>
       </c>
       <c r="F10" t="n">
-        <v>5846.900101238696</v>
+        <v>22993.5927245033</v>
       </c>
       <c r="G10" t="n">
-        <v>-37163.4927360517</v>
+        <v>134.4714820998647</v>
       </c>
       <c r="H10" t="n">
-        <v>84.96184524590689</v>
+        <v>186.7311245683001</v>
       </c>
       <c r="I10" t="n">
-        <v>806.0188355634432</v>
+        <v>1771.486991041363</v>
       </c>
       <c r="J10" t="n">
-        <v>0.2861024355904621</v>
+        <v>-15956.84170861206</v>
       </c>
       <c r="K10" t="n">
-        <v>0.05526627486107727</v>
+        <v>76.35435720685162</v>
       </c>
       <c r="L10" t="n">
-        <v>0.5243019190617298</v>
+        <v>724.3610341552301</v>
+      </c>
+      <c r="M10" t="n">
+        <v>-2168.512970600971</v>
+      </c>
+      <c r="N10" t="n">
+        <v>53.71571108269982</v>
+      </c>
+      <c r="O10" t="n">
+        <v>509.591979470642</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n"/>
+      <c r="A11" s="1" t="n">
+        <v>4</v>
+      </c>
       <c r="B11" s="1" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="C11" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D11" t="n">
-        <v>-432.404009251712</v>
+        <v>-90724.67747501277</v>
       </c>
       <c r="E11" t="n">
-        <v>618.3508780708329</v>
+        <v>2647.842464153626</v>
       </c>
       <c r="F11" t="n">
-        <v>5866.191503606689</v>
+        <v>25119.63921611461</v>
       </c>
       <c r="G11" t="n">
-        <v>-37119.50085467734</v>
+        <v>197.3279063122697</v>
       </c>
       <c r="H11" t="n">
-        <v>77.75195065636878</v>
+        <v>172.3302259327168</v>
       </c>
       <c r="I11" t="n">
-        <v>737.6197697854474</v>
+        <v>1634.8680709164</v>
       </c>
       <c r="J11" t="n">
-        <v>0.2119277228808681</v>
+        <v>-15889.24222445569</v>
       </c>
       <c r="K11" t="n">
-        <v>0.04947247500168624</v>
+        <v>70.71134730650343</v>
       </c>
       <c r="L11" t="n">
-        <v>0.4693371074732129</v>
+        <v>670.8267417232898</v>
+      </c>
+      <c r="M11" t="n">
+        <v>-2123.970966898291</v>
+      </c>
+      <c r="N11" t="n">
+        <v>44.0790990429821</v>
+      </c>
+      <c r="O11" t="n">
+        <v>418.1710505519151</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n"/>
       <c r="B12" s="1" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="C12" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="n">
+        <v>-88806.46643685013</v>
+      </c>
+      <c r="E12" t="n">
+        <v>2361.040651951151</v>
+      </c>
+      <c r="F12" t="n">
+        <v>22398.79832524353</v>
+      </c>
+      <c r="G12" t="n">
+        <v>-192.7715710805742</v>
+      </c>
+      <c r="H12" t="n">
+        <v>170.6684324379681</v>
+      </c>
+      <c r="I12" t="n">
+        <v>1619.102913583629</v>
+      </c>
+      <c r="J12" t="n">
+        <v>-16027.90175697603</v>
+      </c>
+      <c r="K12" t="n">
+        <v>76.24039555870905</v>
+      </c>
+      <c r="L12" t="n">
+        <v>723.2798990331186</v>
+      </c>
+      <c r="M12" t="n">
+        <v>-2074.149666146093</v>
+      </c>
+      <c r="N12" t="n">
+        <v>40.95564520729683</v>
+      </c>
+      <c r="O12" t="n">
+        <v>388.5393656904508</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="n"/>
+      <c r="B13" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C13" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="D12" t="n">
-        <v>470.4832034621473</v>
-      </c>
-      <c r="E12" t="n">
-        <v>630.2037103401099</v>
-      </c>
-      <c r="F12" t="n">
-        <v>5978.637343691261</v>
-      </c>
-      <c r="G12" t="n">
-        <v>-36985.04850914375</v>
-      </c>
-      <c r="H12" t="n">
-        <v>83.90066071722923</v>
-      </c>
-      <c r="I12" t="n">
-        <v>795.9515551783821</v>
-      </c>
-      <c r="J12" t="n">
-        <v>0.1377530198725643</v>
-      </c>
-      <c r="K12" t="n">
-        <v>0.03553692220032265</v>
-      </c>
-      <c r="L12" t="n">
-        <v>0.3371328455556661</v>
+      <c r="D13" t="n">
+        <v>-89883.80103381725</v>
+      </c>
+      <c r="E13" t="n">
+        <v>2620.961319216105</v>
+      </c>
+      <c r="F13" t="n">
+        <v>24864.6222837676</v>
+      </c>
+      <c r="G13" t="n">
+        <v>196.1666294782784</v>
+      </c>
+      <c r="H13" t="n">
+        <v>203.7241559475805</v>
+      </c>
+      <c r="I13" t="n">
+        <v>1932.697041569079</v>
+      </c>
+      <c r="J13" t="n">
+        <v>-16062.90810416363</v>
+      </c>
+      <c r="K13" t="n">
+        <v>72.67709876603197</v>
+      </c>
+      <c r="L13" t="n">
+        <v>689.4754975010214</v>
+      </c>
+      <c r="M13" t="n">
+        <v>-2145.0351830286</v>
+      </c>
+      <c r="N13" t="n">
+        <v>46.78227668645575</v>
+      </c>
+      <c r="O13" t="n">
+        <v>443.8156453721851</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="n"/>
+      <c r="B14" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C14" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" t="n">
+        <v>-96636.71091997848</v>
+      </c>
+      <c r="E14" t="n">
+        <v>2156.105513183136</v>
+      </c>
+      <c r="F14" t="n">
+        <v>20454.61289191473</v>
+      </c>
+      <c r="G14" t="n">
+        <v>386.7617319547859</v>
+      </c>
+      <c r="H14" t="n">
+        <v>209.1031398262767</v>
+      </c>
+      <c r="I14" t="n">
+        <v>1983.7265632311</v>
+      </c>
+      <c r="J14" t="n">
+        <v>-16076.7198885439</v>
+      </c>
+      <c r="K14" t="n">
+        <v>73.4258187101249</v>
+      </c>
+      <c r="L14" t="n">
+        <v>696.5784785598041</v>
+      </c>
+      <c r="M14" t="n">
+        <v>-2056.982574098351</v>
+      </c>
+      <c r="N14" t="n">
+        <v>46.59511135961673</v>
+      </c>
+      <c r="O14" t="n">
+        <v>442.0400391767216</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="n"/>
+      <c r="B15" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="C15" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" t="n">
+        <v>-96991.4117925896</v>
+      </c>
+      <c r="E15" t="n">
+        <v>2414.460394786627</v>
+      </c>
+      <c r="F15" t="n">
+        <v>22905.58250338523</v>
+      </c>
+      <c r="G15" t="n">
+        <v>91.94272286453911</v>
+      </c>
+      <c r="H15" t="n">
+        <v>202.2378723834297</v>
+      </c>
+      <c r="I15" t="n">
+        <v>1918.59691763431</v>
+      </c>
+      <c r="J15" t="n">
+        <v>-15985.5778289316</v>
+      </c>
+      <c r="K15" t="n">
+        <v>75.03121593346189</v>
+      </c>
+      <c r="L15" t="n">
+        <v>711.808613884969</v>
+      </c>
+      <c r="M15" t="n">
+        <v>-2120.221684836697</v>
+      </c>
+      <c r="N15" t="n">
+        <v>45.32388196818793</v>
+      </c>
+      <c r="O15" t="n">
+        <v>429.9800982603273</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="n"/>
+      <c r="B16" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="C16" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" t="n">
+        <v>-91000.54688315019</v>
+      </c>
+      <c r="E16" t="n">
+        <v>2314.564105839029</v>
+      </c>
+      <c r="F16" t="n">
+        <v>21957.88309476708</v>
+      </c>
+      <c r="G16" t="n">
+        <v>62.28135775331832</v>
+      </c>
+      <c r="H16" t="n">
+        <v>171.8793888668086</v>
+      </c>
+      <c r="I16" t="n">
+        <v>1630.591054970708</v>
+      </c>
+      <c r="J16" t="n">
+        <v>-16127.94535908853</v>
+      </c>
+      <c r="K16" t="n">
+        <v>79.4633886912948</v>
+      </c>
+      <c r="L16" t="n">
+        <v>753.8558965792745</v>
+      </c>
+      <c r="M16" t="n">
+        <v>-2094.582745430616</v>
+      </c>
+      <c r="N16" t="n">
+        <v>49.71315701887523</v>
+      </c>
+      <c r="O16" t="n">
+        <v>471.620417571696</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="n"/>
+      <c r="B17" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="C17" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" t="n">
+        <v>-86638.76972263941</v>
+      </c>
+      <c r="E17" t="n">
+        <v>2057.331496830137</v>
+      </c>
+      <c r="F17" t="n">
+        <v>19517.56029596015</v>
+      </c>
+      <c r="G17" t="n">
+        <v>303.1372825694946</v>
+      </c>
+      <c r="H17" t="n">
+        <v>183.1144444567182</v>
+      </c>
+      <c r="I17" t="n">
+        <v>1737.17615087887</v>
+      </c>
+      <c r="J17" t="n">
+        <v>-16112.57390730235</v>
+      </c>
+      <c r="K17" t="n">
+        <v>77.80599157806017</v>
+      </c>
+      <c r="L17" t="n">
+        <v>738.1324469836462</v>
+      </c>
+      <c r="M17" t="n">
+        <v>-2119.467972538846</v>
+      </c>
+      <c r="N17" t="n">
+        <v>50.91773305059004</v>
+      </c>
+      <c r="O17" t="n">
+        <v>483.048029196894</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="n"/>
+      <c r="B18" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="C18" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" t="n">
+        <v>-88845.91511754818</v>
+      </c>
+      <c r="E18" t="n">
+        <v>2355.775978594324</v>
+      </c>
+      <c r="F18" t="n">
+        <v>22348.8532484104</v>
+      </c>
+      <c r="G18" t="n">
+        <v>24.99107272664144</v>
+      </c>
+      <c r="H18" t="n">
+        <v>185.5062936376601</v>
+      </c>
+      <c r="I18" t="n">
+        <v>1759.867224573024</v>
+      </c>
+      <c r="J18" t="n">
+        <v>-16129.49044475534</v>
+      </c>
+      <c r="K18" t="n">
+        <v>72.46876330162246</v>
+      </c>
+      <c r="L18" t="n">
+        <v>687.4990537462523</v>
+      </c>
+      <c r="M18" t="n">
+        <v>-2117.657162855187</v>
+      </c>
+      <c r="N18" t="n">
+        <v>43.00251203086353</v>
+      </c>
+      <c r="O18" t="n">
+        <v>407.9576493789651</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="n"/>
+      <c r="B19" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="C19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" t="n">
+        <v>-87479.56792241994</v>
+      </c>
+      <c r="E19" t="n">
+        <v>2323.80846795565</v>
+      </c>
+      <c r="F19" t="n">
+        <v>22045.58281417878</v>
+      </c>
+      <c r="G19" t="n">
+        <v>238.691235096201</v>
+      </c>
+      <c r="H19" t="n">
+        <v>180.8954416530983</v>
+      </c>
+      <c r="I19" t="n">
+        <v>1716.124841897656</v>
+      </c>
+      <c r="J19" t="n">
+        <v>-16064.65378745947</v>
+      </c>
+      <c r="K19" t="n">
+        <v>76.25435586184226</v>
+      </c>
+      <c r="L19" t="n">
+        <v>723.4123380973004</v>
+      </c>
+      <c r="M19" t="n">
+        <v>-2085.755080792561</v>
+      </c>
+      <c r="N19" t="n">
+        <v>46.84512389920632</v>
+      </c>
+      <c r="O19" t="n">
+        <v>444.41186638284</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A2:A12"/>
+  <mergeCells count="2">
+    <mergeCell ref="A2:A10"/>
+    <mergeCell ref="A11:A19"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>